<commit_message>
Primarily to update the ReadMe file that starts to detail what files do what tasks
</commit_message>
<xml_diff>
--- a/overstory dbh data for 6-9 and 6-6 CAFRI_2023_oct_30.xlsx
+++ b/overstory dbh data for 6-9 and 6-6 CAFRI_2023_oct_30.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjs23\Documents\R\slash-wall-vegetation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BEE7124-30BC-4911-A4FA-FF5CF76B1249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{840A3FDE-E5DC-4402-9577-5E7AE7095574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15252,7 +15252,9 @@
       <c r="D721" s="9">
         <v>833</v>
       </c>
-      <c r="E721" s="9"/>
+      <c r="E721" s="9">
+        <v>634</v>
+      </c>
       <c r="F721" s="10">
         <v>19.3</v>
       </c>
@@ -33274,6 +33276,7 @@
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="9.140625" style="1"/>
+    <col min="6" max="6" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>